<commit_message>
teams fix for team name
</commit_message>
<xml_diff>
--- a/source/teams.xlsx
+++ b/source/teams.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\scygan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BB9BAACF-F0B1-4ADE-978D-C3A26CCFEBD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18C297EA-6E5E-4604-ADCB-2FF9A89FF0FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{EC195DE8-E215-467B-9A6B-FF51D1A76F05}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$95</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -39,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="15">
   <si>
     <t>Season</t>
   </si>
@@ -81,6 +84,9 @@
   </si>
   <si>
     <t>Kiki Owls</t>
+  </si>
+  <si>
+    <t>Gdynia Moustache Admirers</t>
   </si>
 </sst>
 </file>
@@ -452,7 +458,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5129E1F7-3807-4228-B14C-6EA944AEBE0C}">
-  <dimension ref="A1:C95"/>
+  <dimension ref="A1:C96"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="7.42578125" bestFit="1" customWidth="1"/>
@@ -1505,6 +1511,17 @@
         <v>13</v>
       </c>
     </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96">
+        <v>2026</v>
+      </c>
+      <c r="B96">
+        <v>4</v>
+      </c>
+      <c r="C96" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>